<commit_message>
Add institutional v3 Inditex LBO model (100% take-private with Amancio rollover, 2025A-2032E)
</commit_message>
<xml_diff>
--- a/Excels/Inditex_LBO_Ortega_Buyout.xlsx
+++ b/Excels/Inditex_LBO_Ortega_Buyout.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\Escritorio\MEFI\Asignaturas\Módulo 1\Corporate Finance\Inditex LBO\Excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Escritorio\MEFI\Asignaturas\Módulo 1\Corporate Finance\Inditex LBO\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A841AEA9-D84D-4C1B-902C-C28971EE977F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4EFB9C-307C-4D23-9FCA-B2C17F620131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1095,12 +1095,12 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.0_);\(#,##0.0\);&quot;- &quot;"/>
-    <numFmt numFmtId="169" formatCode="0&quot;A&quot;"/>
-    <numFmt numFmtId="171" formatCode="0&quot;E&quot;"/>
-    <numFmt numFmtId="173" formatCode="#,##0.0%_);\(#,##0.0%\);&quot;- &quot;"/>
-    <numFmt numFmtId="176" formatCode="0.0"/>
-    <numFmt numFmtId="187" formatCode="#,##0.0&quot;x&quot;_);\(#,##0.0&quot;x&quot;\);&quot;- &quot;"/>
-    <numFmt numFmtId="188" formatCode="#,##0.00_);\(#,##0.00\);&quot;- &quot;"/>
+    <numFmt numFmtId="165" formatCode="0&quot;A&quot;"/>
+    <numFmt numFmtId="166" formatCode="0&quot;E&quot;"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0%_);\(#,##0.0%\);&quot;- &quot;"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0&quot;x&quot;_);\(#,##0.0&quot;x&quot;\);&quot;- &quot;"/>
+    <numFmt numFmtId="170" formatCode="#,##0.00_);\(#,##0.00\);&quot;- &quot;"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -1337,10 +1337,10 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1354,67 +1354,67 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="173" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="173" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="173" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="7" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="173" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="11" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="173" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="173" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="187" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="188" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="188" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1423,7 +1423,7 @@
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1432,46 +1432,46 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="187" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="7" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="173" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="187" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="15" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="187" fontId="7" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="7" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="187" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="173" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1837,7 +1837,7 @@
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="4" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="4" max="4" width="83.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="90" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
@@ -3411,19 +3411,19 @@
       </c>
       <c r="O34" s="29">
         <f>+O133</f>
-        <v>-3879.9452671618747</v>
+        <v>-3952.8593704382497</v>
       </c>
       <c r="P34" s="29">
         <f>+P133</f>
-        <v>-3792.3117715487497</v>
+        <v>-3943.7908211054187</v>
       </c>
       <c r="Q34" s="29">
         <f>+Q133</f>
-        <v>-3680.3079602504713</v>
+        <v>-3915.7729135055602</v>
       </c>
       <c r="R34" s="29">
         <f>+R133</f>
-        <v>-3542.5484046666188</v>
+        <v>-3869.2775283472711</v>
       </c>
     </row>
     <row r="35" spans="2:22" x14ac:dyDescent="0.2">
@@ -3452,19 +3452,19 @@
       </c>
       <c r="O35" s="41">
         <f t="shared" si="16"/>
-        <v>2111.0220600763951</v>
+        <v>2038.10795680002</v>
       </c>
       <c r="P35" s="41">
         <f t="shared" si="16"/>
-        <v>2580.1369661116396</v>
+        <v>2428.6579165549706</v>
       </c>
       <c r="Q35" s="41">
         <f t="shared" si="16"/>
-        <v>3099.9046188188677</v>
+        <v>2864.4396655637788</v>
       </c>
       <c r="R35" s="41">
         <f t="shared" si="16"/>
-        <v>3673.3619331572827</v>
+        <v>3346.6328094766304</v>
       </c>
       <c r="U35" s="30">
         <f>+IFERROR((M35/J35)^(1/(M$20-J$20))-1,0)</f>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="V35" s="30">
         <f>+IFERROR((R35/M35)^(1/(R$20-M$20))-1,"n.a.")</f>
-        <v>-6.00844495688313E-2</v>
+        <v>-7.7433451260560671E-2</v>
       </c>
     </row>
     <row r="36" spans="2:22" x14ac:dyDescent="0.2">
@@ -3500,19 +3500,19 @@
       </c>
       <c r="O36" s="34">
         <f>+IF(O35&gt;0,-O35*$F$36,0)</f>
-        <v>-472.8689414571125</v>
+        <v>-456.53618232320451</v>
       </c>
       <c r="P36" s="34">
         <f>+IF(P35&gt;0,-P35*$F$36,0)</f>
-        <v>-577.9506804090073</v>
+        <v>-544.01937330831345</v>
       </c>
       <c r="Q36" s="34">
         <f>+IF(Q35&gt;0,-Q35*$F$36,0)</f>
-        <v>-694.37863461542634</v>
+        <v>-641.63448508628642</v>
       </c>
       <c r="R36" s="34">
         <f>+IF(R35&gt;0,-R35*$F$36,0)</f>
-        <v>-822.83307302723131</v>
+        <v>-749.64574932276525</v>
       </c>
       <c r="U36" s="30">
         <f>+IFERROR((M36/J36)^(1/(M$20-J$20))-1,0)</f>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="V36" s="30">
         <f>+IFERROR((R36/M36)^(1/(R$20-M$20))-1,"n.a.")</f>
-        <v>-6.6088688120411576E-2</v>
+        <v>-8.3326863318482824E-2</v>
       </c>
     </row>
     <row r="37" spans="2:22" x14ac:dyDescent="0.2">
@@ -3554,19 +3554,19 @@
       </c>
       <c r="O37" s="36">
         <f t="shared" si="17"/>
-        <v>1638.1531186192826</v>
+        <v>1581.5717744768156</v>
       </c>
       <c r="P37" s="36">
         <f t="shared" si="17"/>
-        <v>2002.1862857026322</v>
+        <v>1884.6385432466573</v>
       </c>
       <c r="Q37" s="36">
         <f t="shared" si="17"/>
-        <v>2405.5259842034411</v>
+        <v>2222.8051804774923</v>
       </c>
       <c r="R37" s="36">
         <f t="shared" si="17"/>
-        <v>2850.5288601300513</v>
+        <v>2596.9870601538651</v>
       </c>
       <c r="S37" s="35"/>
       <c r="T37" s="35"/>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="V37" s="37">
         <f>+IFERROR((R37/M37)^(1/(R$20-M$20))-1,"n.a.")</f>
-        <v>-5.8307517086756633E-2</v>
+        <v>-7.5689317474734286E-2</v>
       </c>
     </row>
     <row r="40" spans="2:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -4873,19 +4873,19 @@
       </c>
       <c r="O97" s="34">
         <f>+N101</f>
-        <v>12139.705019999999</v>
+        <v>13080.532159049999</v>
       </c>
       <c r="P97" s="34">
         <f>+O101</f>
-        <v>12139.705019999999</v>
+        <v>14094.273401376373</v>
       </c>
       <c r="Q97" s="34">
         <f>+P101</f>
-        <v>12139.705019999999</v>
+        <v>15186.579589983041</v>
       </c>
       <c r="R97" s="34">
         <f>+Q101</f>
-        <v>12139.705019999999</v>
+        <v>16363.539508206726</v>
       </c>
     </row>
     <row r="98" spans="4:18" x14ac:dyDescent="0.2">
@@ -4921,23 +4921,23 @@
       </c>
       <c r="N99" s="34">
         <f>+IF($I$180=1,N97*$F$180,0)</f>
-        <v>0</v>
+        <v>940.82713904999991</v>
       </c>
       <c r="O99" s="34">
         <f>+IF($I$180=1,O97*$F$180,0)</f>
-        <v>0</v>
+        <v>1013.741242326375</v>
       </c>
       <c r="P99" s="34">
         <f>+IF($I$180=1,P97*$F$180,0)</f>
-        <v>0</v>
+        <v>1092.3061886066689</v>
       </c>
       <c r="Q99" s="34">
         <f>+IF($I$180=1,Q97*$F$180,0)</f>
-        <v>0</v>
+        <v>1176.9599182236857</v>
       </c>
       <c r="R99" s="34">
         <f>+IF($I$180=1,R97*$F$180,0)</f>
-        <v>0</v>
+        <v>1268.1743118860213</v>
       </c>
     </row>
     <row r="100" spans="4:18" x14ac:dyDescent="0.2">
@@ -4981,23 +4981,23 @@
       </c>
       <c r="N101" s="27">
         <f t="shared" si="27"/>
-        <v>12139.705019999999</v>
+        <v>13080.532159049999</v>
       </c>
       <c r="O101" s="27">
         <f t="shared" si="27"/>
-        <v>12139.705019999999</v>
+        <v>14094.273401376373</v>
       </c>
       <c r="P101" s="27">
         <f t="shared" si="27"/>
-        <v>12139.705019999999</v>
+        <v>15186.579589983041</v>
       </c>
       <c r="Q101" s="27">
         <f t="shared" si="27"/>
-        <v>12139.705019999999</v>
+        <v>16363.539508206726</v>
       </c>
       <c r="R101" s="27">
         <f t="shared" si="27"/>
-        <v>12139.705019999999</v>
+        <v>17631.713820092747</v>
       </c>
     </row>
     <row r="102" spans="4:18" x14ac:dyDescent="0.2">
@@ -5006,23 +5006,23 @@
       </c>
       <c r="N102" s="34">
         <f>+IF($I$180=0,-N97*$F$180,0)</f>
-        <v>-940.82713904999991</v>
+        <v>0</v>
       </c>
       <c r="O102" s="34">
         <f>+IF($I$180=0,-O97*$F$180,0)</f>
-        <v>-940.82713904999991</v>
+        <v>0</v>
       </c>
       <c r="P102" s="34">
         <f>+IF($I$180=0,-P97*$F$180,0)</f>
-        <v>-940.82713904999991</v>
+        <v>0</v>
       </c>
       <c r="Q102" s="34">
         <f>+IF($I$180=0,-Q97*$F$180,0)</f>
-        <v>-940.82713904999991</v>
+        <v>0</v>
       </c>
       <c r="R102" s="34">
         <f>+IF($I$180=0,-R97*$F$180,0)</f>
-        <v>-940.82713904999991</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" spans="4:18" x14ac:dyDescent="0.2">
@@ -5035,19 +5035,19 @@
       </c>
       <c r="O103" s="39">
         <f>-O97*$F$180</f>
-        <v>-940.82713904999991</v>
+        <v>-1013.741242326375</v>
       </c>
       <c r="P103" s="39">
         <f>-P97*$F$180</f>
-        <v>-940.82713904999991</v>
+        <v>-1092.3061886066689</v>
       </c>
       <c r="Q103" s="39">
         <f>-Q97*$F$180</f>
-        <v>-940.82713904999991</v>
+        <v>-1176.9599182236857</v>
       </c>
       <c r="R103" s="39">
         <f>-R97*$F$180</f>
-        <v>-940.82713904999991</v>
+        <v>-1268.1743118860213</v>
       </c>
     </row>
     <row r="105" spans="4:18" x14ac:dyDescent="0.2">
@@ -5271,11 +5271,11 @@
       </c>
       <c r="Q115" s="34">
         <f>+P117</f>
-        <v>13.629100379530882</v>
+        <v>0</v>
       </c>
       <c r="R115" s="34">
         <f>+Q117</f>
-        <v>12.613248068758821</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116" spans="4:18" x14ac:dyDescent="0.2">
@@ -5296,15 +5296,15 @@
       </c>
       <c r="P116" s="34">
         <f>+IF(P150&lt;0,MIN($F$184-P115,-P150),-MIN(P115,P150))</f>
-        <v>13.629100379530882</v>
+        <v>0</v>
       </c>
       <c r="Q116" s="34">
         <f>+IF(Q150&lt;0,MIN($F$184-Q115,-Q150),-MIN(Q115,Q150))</f>
-        <v>-1.0158523107720612</v>
+        <v>0</v>
       </c>
       <c r="R116" s="34">
         <f>+IF(R150&lt;0,MIN($F$184-R115,-R150),-MIN(R115,R150))</f>
-        <v>-12.613248068758821</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117" spans="4:18" x14ac:dyDescent="0.2">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="P117" s="27">
         <f t="shared" si="29"/>
-        <v>13.629100379530882</v>
+        <v>0</v>
       </c>
       <c r="Q117" s="27">
         <f t="shared" si="29"/>
-        <v>12.613248068758821</v>
+        <v>0</v>
       </c>
       <c r="R117" s="27">
         <f t="shared" si="29"/>
@@ -5362,11 +5362,11 @@
       </c>
       <c r="P118" s="39">
         <f>+MAX(0,$F$184-P117)</f>
-        <v>1986.3708996204691</v>
+        <v>2000</v>
       </c>
       <c r="Q118" s="39">
         <f>+MAX(0,$F$184-Q117)</f>
-        <v>1987.3867519312412</v>
+        <v>2000</v>
       </c>
       <c r="R118" s="39">
         <f>+MAX(0,$F$184-R117)</f>
@@ -5391,11 +5391,11 @@
       </c>
       <c r="Q119" s="34">
         <f>-(Q115*$F$185+MAX(0,$F$184-Q115)*$F$186)</f>
-        <v>-7.6678259185970132</v>
+        <v>-7</v>
       </c>
       <c r="R119" s="34">
         <f>-(R115*$F$185+MAX(0,$F$184-R115)*$F$186)</f>
-        <v>-7.6180491553691825</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="126" spans="4:18" x14ac:dyDescent="0.2">
@@ -5416,19 +5416,19 @@
       </c>
       <c r="O127" s="34">
         <f>+O79+O87+O97+O106+O115</f>
-        <v>62822.973478500004</v>
+        <v>63763.800617550005</v>
       </c>
       <c r="P127" s="34">
         <f>+P79+P87+P97+P106+P115</f>
-        <v>61457.256663749999</v>
+        <v>63411.825045126374</v>
       </c>
       <c r="Q127" s="34">
         <f>+Q79+Q87+Q97+Q106+Q115</f>
-        <v>59649.930011129531</v>
+        <v>62683.175480733044</v>
       </c>
       <c r="R127" s="34">
         <f>+R79+R87+R97+R106+R115</f>
-        <v>57372.719467568757</v>
+        <v>61583.94070770673</v>
       </c>
     </row>
     <row r="128" spans="4:18" x14ac:dyDescent="0.2">
@@ -5477,15 +5477,15 @@
       </c>
       <c r="P129" s="34">
         <f>+P91+P116</f>
-        <v>13.629100379530882</v>
+        <v>0</v>
       </c>
       <c r="Q129" s="34">
         <f>+Q91+Q116</f>
-        <v>-1.0158523107720612</v>
+        <v>0</v>
       </c>
       <c r="R129" s="34">
         <f>+R91+R116</f>
-        <v>-12.613248068758821</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130" spans="2:22" x14ac:dyDescent="0.2">
@@ -5497,23 +5497,23 @@
       </c>
       <c r="N130" s="34">
         <f>+N99+N108</f>
-        <v>0</v>
+        <v>940.82713904999991</v>
       </c>
       <c r="O130" s="34">
         <f>+O99+O108</f>
-        <v>0</v>
+        <v>1013.741242326375</v>
       </c>
       <c r="P130" s="34">
         <f>+P99+P108</f>
-        <v>0</v>
+        <v>1092.3061886066689</v>
       </c>
       <c r="Q130" s="34">
         <f>+Q99+Q108</f>
-        <v>0</v>
+        <v>1176.9599182236857</v>
       </c>
       <c r="R130" s="34">
         <f>+R99+R108</f>
-        <v>0</v>
+        <v>1268.1743118860213</v>
       </c>
     </row>
     <row r="131" spans="2:22" x14ac:dyDescent="0.2">
@@ -5534,23 +5534,23 @@
       </c>
       <c r="N131" s="36">
         <f t="shared" si="30"/>
-        <v>62822.973478500004</v>
+        <v>63763.800617550005</v>
       </c>
       <c r="O131" s="36">
         <f t="shared" si="30"/>
-        <v>61457.256663749999</v>
+        <v>63411.825045126374</v>
       </c>
       <c r="P131" s="36">
         <f t="shared" si="30"/>
-        <v>59649.930011129531</v>
+        <v>62683.175480733044</v>
       </c>
       <c r="Q131" s="36">
         <f t="shared" si="30"/>
-        <v>57372.719467568757</v>
+        <v>61583.94070770673</v>
       </c>
       <c r="R131" s="36">
         <f t="shared" si="30"/>
-        <v>54628.672590000002</v>
+        <v>60120.681390092752</v>
       </c>
     </row>
     <row r="132" spans="2:22" x14ac:dyDescent="0.2">
@@ -5559,23 +5559,23 @@
       </c>
       <c r="N132" s="41">
         <f>+N84+N94+N102+N111+N119</f>
-        <v>-3942.5406211712493</v>
+        <v>-3001.7134821212494</v>
       </c>
       <c r="O132" s="41">
         <f>+O84+O94+O102+O111+O119</f>
-        <v>-3879.9452671618747</v>
+        <v>-2939.1181281118747</v>
       </c>
       <c r="P132" s="41">
         <f>+P84+P94+P102+P111+P119</f>
-        <v>-3792.3117715487497</v>
+        <v>-2851.4846324987498</v>
       </c>
       <c r="Q132" s="41">
         <f>+Q84+Q94+Q102+Q111+Q119</f>
-        <v>-3680.3079602504713</v>
+        <v>-2738.8129952818745</v>
       </c>
       <c r="R132" s="41">
         <f>+R84+R94+R102+R111+R119</f>
-        <v>-3542.5484046666188</v>
+        <v>-2601.1032164612498</v>
       </c>
     </row>
     <row r="133" spans="2:22" x14ac:dyDescent="0.2">
@@ -5588,19 +5588,19 @@
       </c>
       <c r="O133" s="39">
         <f>+O84+O94+O103+O112+O119</f>
-        <v>-3879.9452671618747</v>
+        <v>-3952.8593704382497</v>
       </c>
       <c r="P133" s="39">
         <f>+P84+P94+P103+P112+P119</f>
-        <v>-3792.3117715487497</v>
+        <v>-3943.7908211054187</v>
       </c>
       <c r="Q133" s="39">
         <f>+Q84+Q94+Q103+Q112+Q119</f>
-        <v>-3680.3079602504713</v>
+        <v>-3915.7729135055602</v>
       </c>
       <c r="R133" s="39">
         <f>+R84+R94+R103+R112+R119</f>
-        <v>-3542.5484046666188</v>
+        <v>-3869.2775283472711</v>
       </c>
     </row>
     <row r="134" spans="2:22" x14ac:dyDescent="0.2">
@@ -5613,23 +5613,23 @@
       </c>
       <c r="N134" s="54">
         <f t="shared" si="31"/>
-        <v>3.8426892611253618</v>
+        <v>3.698540915174529</v>
       </c>
       <c r="O134" s="54">
         <f t="shared" si="31"/>
-        <v>3.3769799181555418</v>
+        <v>3.1069248284420197</v>
       </c>
       <c r="P134" s="54">
         <f t="shared" si="31"/>
-        <v>2.9017943161306614</v>
+        <v>2.5219107935558855</v>
       </c>
       <c r="Q134" s="54">
         <f t="shared" si="31"/>
-        <v>2.4187639516223136</v>
+        <v>1.9431712047792411</v>
       </c>
       <c r="R134" s="54">
         <f t="shared" si="31"/>
-        <v>1.9294089061995903</v>
+        <v>1.3706386659042678</v>
       </c>
     </row>
     <row r="135" spans="2:22" x14ac:dyDescent="0.2">
@@ -5642,23 +5642,23 @@
       </c>
       <c r="N135" s="54">
         <f t="shared" si="32"/>
-        <v>9.4226252334156619</v>
+        <v>9.4226252334156637</v>
       </c>
       <c r="O135" s="54">
         <f t="shared" si="32"/>
-        <v>8.5588737835367112</v>
+        <v>8.5669244602108652</v>
       </c>
       <c r="P135" s="54">
         <f t="shared" si="32"/>
-        <v>7.717752359774944</v>
+        <v>7.7407786846555631</v>
       </c>
       <c r="Q135" s="54">
         <f t="shared" si="32"/>
-        <v>6.8978784995479883</v>
+        <v>6.9417667580228137</v>
       </c>
       <c r="R135" s="54">
         <f t="shared" si="32"/>
-        <v>6.0980926058282909</v>
+        <v>6.167960582728683</v>
       </c>
     </row>
     <row r="138" spans="2:22" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -5824,19 +5824,19 @@
       </c>
       <c r="O142" s="34">
         <f t="shared" si="35"/>
-        <v>-472.8689414571125</v>
+        <v>-456.53618232320451</v>
       </c>
       <c r="P142" s="34">
         <f t="shared" si="35"/>
-        <v>-577.9506804090073</v>
+        <v>-544.01937330831345</v>
       </c>
       <c r="Q142" s="34">
         <f t="shared" si="35"/>
-        <v>-694.37863461542634</v>
+        <v>-641.63448508628642</v>
       </c>
       <c r="R142" s="34">
         <f t="shared" si="35"/>
-        <v>-822.83307302723131</v>
+        <v>-749.64574932276525</v>
       </c>
     </row>
     <row r="143" spans="2:22" x14ac:dyDescent="0.2">
@@ -5952,19 +5952,19 @@
       </c>
       <c r="O145" s="27">
         <f t="shared" si="38"/>
-        <v>5226.4885416162397</v>
+        <v>5242.8213007501472</v>
       </c>
       <c r="P145" s="27">
         <f t="shared" si="38"/>
-        <v>5582.3502099342741</v>
+        <v>5616.2815170349677</v>
       </c>
       <c r="Q145" s="27">
         <f t="shared" si="38"/>
-        <v>5957.5185038112431</v>
+        <v>6010.2626533403836</v>
       </c>
       <c r="R145" s="27">
         <f t="shared" si="38"/>
-        <v>6353.2050131955348</v>
+        <v>6426.3923369000004</v>
       </c>
     </row>
     <row r="147" spans="1:22" x14ac:dyDescent="0.2">
@@ -5973,23 +5973,23 @@
       </c>
       <c r="N147" s="34">
         <f>+N132</f>
-        <v>-3942.5406211712493</v>
+        <v>-3001.7134821212494</v>
       </c>
       <c r="O147" s="34">
         <f>+O132</f>
-        <v>-3879.9452671618747</v>
+        <v>-2939.1181281118747</v>
       </c>
       <c r="P147" s="34">
         <f>+P132</f>
-        <v>-3792.3117715487497</v>
+        <v>-2851.4846324987498</v>
       </c>
       <c r="Q147" s="34">
         <f>+Q132</f>
-        <v>-3680.3079602504713</v>
+        <v>-2738.8129952818745</v>
       </c>
       <c r="R147" s="34">
         <f>+R132</f>
-        <v>-3542.5484046666188</v>
+        <v>-2601.1032164612498</v>
       </c>
     </row>
     <row r="148" spans="1:22" x14ac:dyDescent="0.2">
@@ -6032,23 +6032,23 @@
       <c r="M149" s="17"/>
       <c r="N149" s="27">
         <f>+N145+N147+N148</f>
-        <v>36.461754530579697</v>
+        <v>977.28889358057961</v>
       </c>
       <c r="O149" s="27">
         <f>+O145+O147+O148</f>
-        <v>-19.173540295634893</v>
+        <v>937.98635788827255</v>
       </c>
       <c r="P149" s="27">
         <f>+P145+P147+P148</f>
-        <v>-30.917314614475572</v>
+        <v>943.84113153621797</v>
       </c>
       <c r="Q149" s="27">
         <f>+Q145+Q147+Q148</f>
-        <v>1.0158523107720612</v>
+        <v>995.25496680850938</v>
       </c>
       <c r="R149" s="27">
         <f>+R145+R147+R148</f>
-        <v>79.222979028915688</v>
+        <v>1093.8554909387503</v>
       </c>
     </row>
     <row r="150" spans="1:22" x14ac:dyDescent="0.2">
@@ -6057,23 +6057,23 @@
       </c>
       <c r="N150" s="39">
         <f>+(N156-$F$171*$F$168)+N149</f>
-        <v>36.461754530579697</v>
+        <v>977.28889358057961</v>
       </c>
       <c r="O150" s="39">
         <f>+(O156-$F$171*$F$168)+O149</f>
-        <v>17.288214234944689</v>
+        <v>1915.275251468852</v>
       </c>
       <c r="P150" s="39">
         <f>+(P156-$F$171*$F$168)+P149</f>
-        <v>-13.629100379530882</v>
+        <v>2859.11638300507</v>
       </c>
       <c r="Q150" s="39">
         <f>+(Q156-$F$171*$F$168)+Q149</f>
-        <v>1.0158523107720612</v>
+        <v>3854.3713498135799</v>
       </c>
       <c r="R150" s="39">
         <f>+(R156-$F$171*$F$168)+R149</f>
-        <v>79.222979028915688</v>
+        <v>4948.2268407523297</v>
       </c>
     </row>
     <row r="151" spans="1:22" x14ac:dyDescent="0.2">
@@ -6090,15 +6090,15 @@
       </c>
       <c r="P151" s="34">
         <f>+P116</f>
-        <v>13.629100379530882</v>
+        <v>0</v>
       </c>
       <c r="Q151" s="34">
         <f>+Q116</f>
-        <v>-1.0158523107720612</v>
+        <v>0</v>
       </c>
       <c r="R151" s="34">
         <f>+R116</f>
-        <v>-12.613248068758821</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:22" x14ac:dyDescent="0.2">
@@ -6161,23 +6161,23 @@
       <c r="M154" s="17"/>
       <c r="N154" s="27">
         <f>+N149+SUM(N151:N153)</f>
-        <v>36.461754530579697</v>
+        <v>977.28889358057961</v>
       </c>
       <c r="O154" s="27">
         <f>+O149+SUM(O151:O153)</f>
-        <v>-19.173540295634893</v>
+        <v>937.98635788827255</v>
       </c>
       <c r="P154" s="27">
         <f>+P149+SUM(P151:P153)</f>
-        <v>-17.288214234944689</v>
+        <v>943.84113153621797</v>
       </c>
       <c r="Q154" s="27">
         <f>+Q149+SUM(Q151:Q153)</f>
-        <v>0</v>
+        <v>995.25496680850938</v>
       </c>
       <c r="R154" s="27">
         <f>+R149+SUM(R151:R153)</f>
-        <v>66.609730960156867</v>
+        <v>1093.8554909387503</v>
       </c>
     </row>
     <row r="156" spans="1:22" x14ac:dyDescent="0.2">
@@ -6194,19 +6194,19 @@
       </c>
       <c r="O156" s="34">
         <f>+N157</f>
-        <v>1323.4017545305796</v>
+        <v>2264.2288935805796</v>
       </c>
       <c r="P156" s="34">
         <f>+O157</f>
-        <v>1304.2282142349447</v>
+        <v>3202.2152514688523</v>
       </c>
       <c r="Q156" s="34">
         <f>+P157</f>
-        <v>1286.94</v>
+        <v>4146.0563830050705</v>
       </c>
       <c r="R156" s="34">
         <f>+Q157</f>
-        <v>1286.94</v>
+        <v>5141.3113498135799</v>
       </c>
     </row>
     <row r="157" spans="1:22" x14ac:dyDescent="0.2">
@@ -6227,23 +6227,23 @@
       </c>
       <c r="N157" s="36">
         <f>+N156+N154</f>
-        <v>1323.4017545305796</v>
+        <v>2264.2288935805796</v>
       </c>
       <c r="O157" s="36">
         <f>+O156+O154</f>
-        <v>1304.2282142349447</v>
+        <v>3202.2152514688523</v>
       </c>
       <c r="P157" s="36">
         <f>+P156+P154</f>
-        <v>1286.94</v>
+        <v>4146.0563830050705</v>
       </c>
       <c r="Q157" s="36">
         <f>+Q156+Q154</f>
-        <v>1286.94</v>
+        <v>5141.3113498135799</v>
       </c>
       <c r="R157" s="36">
         <f>+R156+R154</f>
-        <v>1353.5497309601569</v>
+        <v>6235.1668407523302</v>
       </c>
     </row>
     <row r="160" spans="1:22" ht="16.05" customHeight="1" x14ac:dyDescent="0.2">
@@ -6536,7 +6536,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
       <c r="I180" s="70">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="181" spans="2:22" x14ac:dyDescent="0.2">
@@ -7055,23 +7055,23 @@
       </c>
       <c r="N218" s="34">
         <f>-N131</f>
-        <v>-62822.973478500004</v>
+        <v>-63763.800617550005</v>
       </c>
       <c r="O218" s="34">
         <f>-O131</f>
-        <v>-61457.256663749999</v>
+        <v>-63411.825045126374</v>
       </c>
       <c r="P218" s="34">
         <f>-P131</f>
-        <v>-59649.930011129531</v>
+        <v>-62683.175480733044</v>
       </c>
       <c r="Q218" s="34">
         <f>-Q131</f>
-        <v>-57372.719467568757</v>
+        <v>-61583.94070770673</v>
       </c>
       <c r="R218" s="34">
         <f>-R131</f>
-        <v>-54628.672590000002</v>
+        <v>-60120.681390092752</v>
       </c>
     </row>
     <row r="219" spans="2:22" x14ac:dyDescent="0.2">
@@ -7080,23 +7080,23 @@
       </c>
       <c r="N219" s="34">
         <f>+N157</f>
-        <v>1323.4017545305796</v>
+        <v>2264.2288935805796</v>
       </c>
       <c r="O219" s="34">
         <f>+O157</f>
-        <v>1304.2282142349447</v>
+        <v>3202.2152514688523</v>
       </c>
       <c r="P219" s="34">
         <f>+P157</f>
-        <v>1286.94</v>
+        <v>4146.0563830050705</v>
       </c>
       <c r="Q219" s="34">
         <f>+Q157</f>
-        <v>1286.94</v>
+        <v>5141.3113498135799</v>
       </c>
       <c r="R219" s="34">
         <f>+R157</f>
-        <v>1353.5497309601569</v>
+        <v>6235.1668407523302</v>
       </c>
     </row>
     <row r="220" spans="2:22" x14ac:dyDescent="0.2">
@@ -7164,23 +7164,23 @@
       <c r="M222" s="35"/>
       <c r="N222" s="36">
         <f>+SUM(N217:N221)</f>
-        <v>55814.714315808895</v>
+        <v>55814.714315808887</v>
       </c>
       <c r="O222" s="36">
         <f>+SUM(O217:O221)</f>
-        <v>66172.639683165107</v>
+        <v>66116.058339022638</v>
       </c>
       <c r="P222" s="36">
         <f>+SUM(P217:P221)</f>
-        <v>77561.409413572648</v>
+        <v>77387.2803269742</v>
       </c>
       <c r="Q222" s="36">
         <f>+SUM(Q217:Q221)</f>
-        <v>90060.562121321345</v>
+        <v>89703.712230996956</v>
       </c>
       <c r="R222" s="36">
         <f>+SUM(R217:R221)</f>
-        <v>103754.35020825425</v>
+        <v>103143.95851795367</v>
       </c>
     </row>
     <row r="224" spans="2:22" x14ac:dyDescent="0.2">
@@ -7214,23 +7214,23 @@
       </c>
       <c r="N225" s="41">
         <f>+N222*$F$208</f>
-        <v>55814.714315808895</v>
+        <v>55814.714315808887</v>
       </c>
       <c r="O225" s="41">
         <f>+O222*$F$208</f>
-        <v>66172.639683165107</v>
+        <v>66116.058339022638</v>
       </c>
       <c r="P225" s="41">
         <f>+P222*$F$208</f>
-        <v>77561.409413572648</v>
+        <v>77387.2803269742</v>
       </c>
       <c r="Q225" s="41">
         <f>+Q222*$F$208</f>
-        <v>90060.562121321345</v>
+        <v>89703.712230996956</v>
       </c>
       <c r="R225" s="41">
         <f>+R222*$F$208</f>
-        <v>103754.35020825425</v>
+        <v>103143.95851795367</v>
       </c>
     </row>
     <row r="227" spans="4:22" x14ac:dyDescent="0.2">
@@ -7245,7 +7245,7 @@
       <c r="E229" s="77"/>
       <c r="F229" s="78">
         <f>+INDEX(U235:U239,MATCH($K$166,D235:D239,0))</f>
-        <v>0.15922031998634348</v>
+        <v>0.15785389542579656</v>
       </c>
       <c r="N229" s="74">
         <f>+U235</f>
@@ -7253,19 +7253,19 @@
       </c>
       <c r="O229" s="74">
         <f>+U236</f>
-        <v>0.15568355917930607</v>
+        <v>0.15518936514854434</v>
       </c>
       <c r="P229" s="74">
         <f>+U237</f>
-        <v>0.1609740197658539</v>
+        <v>0.16010535359382633</v>
       </c>
       <c r="Q229" s="74">
         <f>+U238</f>
-        <v>0.16101841330528263</v>
+        <v>0.159867399930954</v>
       </c>
       <c r="R229" s="74">
         <f>+U239</f>
-        <v>0.15922031998634348</v>
+        <v>0.15785389542579656</v>
       </c>
     </row>
     <row r="230" spans="4:22" x14ac:dyDescent="0.2">
@@ -7275,7 +7275,7 @@
       <c r="E230" s="77"/>
       <c r="F230" s="79">
         <f>+INDEX(V235:V239,MATCH($K$166,D235:D239,0))</f>
-        <v>2.0941400700990314</v>
+        <v>2.0818201462158563</v>
       </c>
       <c r="N230" s="66">
         <f>+V235</f>
@@ -7283,19 +7283,19 @@
       </c>
       <c r="O230" s="66">
         <f>+V236</f>
-        <v>1.335604492983629</v>
+        <v>1.3344624757115726</v>
       </c>
       <c r="P230" s="66">
         <f>+V237</f>
-        <v>1.5654712792312093</v>
+        <v>1.561956721076456</v>
       </c>
       <c r="Q230" s="66">
         <f>+V238</f>
-        <v>1.8177496316573516</v>
+        <v>1.8105471032540723</v>
       </c>
       <c r="R230" s="66">
         <f>+V239</f>
-        <v>2.0941400700990314</v>
+        <v>2.0818201462158563</v>
       </c>
     </row>
     <row r="232" spans="4:22" x14ac:dyDescent="0.2">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="N235" s="34">
         <f>+(IF($D235=N$234,N$222,0)+N$220)*$F$208</f>
-        <v>55814.714315808895</v>
+        <v>55814.714315808887</v>
       </c>
       <c r="O235" s="34">
         <v>0</v>
@@ -7452,7 +7452,7 @@
       </c>
       <c r="O236" s="34">
         <f>+(IF($D236=O$234,O$222,0)+O$220)*$F$208</f>
-        <v>66172.639683165107</v>
+        <v>66116.058339022638</v>
       </c>
       <c r="P236" s="34">
         <v>0</v>
@@ -7465,11 +7465,11 @@
       </c>
       <c r="U236" s="74">
         <f>+IFERROR(XIRR(M236:O236,$M$232:$O$232),0)</f>
-        <v>0.15568355917930607</v>
+        <v>0.15518936514854434</v>
       </c>
       <c r="V236" s="66">
         <f>-SUM(N236:O236)/M236</f>
-        <v>1.335604492983629</v>
+        <v>1.3344624757115726</v>
       </c>
     </row>
     <row r="237" spans="4:22" x14ac:dyDescent="0.2">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="P237" s="34">
         <f>+(IF($D237=P$234,P$222,0)+P$220)*$F$208</f>
-        <v>77561.409413572648</v>
+        <v>77387.2803269742</v>
       </c>
       <c r="Q237" s="34">
         <v>0</v>
@@ -7501,11 +7501,11 @@
       </c>
       <c r="U237" s="74">
         <f>+IFERROR(XIRR(M237:P237,$M$232:$P$232),0)</f>
-        <v>0.1609740197658539</v>
+        <v>0.16010535359382633</v>
       </c>
       <c r="V237" s="66">
         <f>-SUM(N237:P237)/M237</f>
-        <v>1.5654712792312093</v>
+        <v>1.561956721076456</v>
       </c>
     </row>
     <row r="238" spans="4:22" x14ac:dyDescent="0.2">
@@ -7531,18 +7531,18 @@
       </c>
       <c r="Q238" s="34">
         <f>+(IF($D238=Q$234,Q$222,0)+Q$220)*$F$208</f>
-        <v>90060.562121321345</v>
+        <v>89703.712230996956</v>
       </c>
       <c r="R238" s="34">
         <v>0</v>
       </c>
       <c r="U238" s="74">
         <f>+IFERROR(XIRR(M238:Q238,$M$232:$Q$232),0)</f>
-        <v>0.16101841330528263</v>
+        <v>0.159867399930954</v>
       </c>
       <c r="V238" s="66">
         <f>-SUM(N238:Q238)/M238</f>
-        <v>1.8177496316573516</v>
+        <v>1.8105471032540723</v>
       </c>
     </row>
     <row r="239" spans="4:22" x14ac:dyDescent="0.2">
@@ -7572,15 +7572,15 @@
       </c>
       <c r="R239" s="34">
         <f>+(IF($D239=R$234,R$222,0)+R$220)*$F$208</f>
-        <v>103754.35020825425</v>
+        <v>103143.95851795367</v>
       </c>
       <c r="U239" s="74">
         <f>+IFERROR(XIRR(M239:R239,$M$232:$R$232),0)</f>
-        <v>0.15922031998634348</v>
+        <v>0.15785389542579656</v>
       </c>
       <c r="V239" s="66">
         <f>-SUM(N239:R239)/M239</f>
-        <v>2.0941400700990314</v>
+        <v>2.0818201462158563</v>
       </c>
     </row>
     <row r="241" spans="2:22" x14ac:dyDescent="0.2">
@@ -7618,17 +7618,17 @@
       </c>
       <c r="R241" s="36">
         <f t="shared" si="42"/>
-        <v>103754.35020825425</v>
+        <v>103143.95851795367</v>
       </c>
       <c r="S241" s="35"/>
       <c r="T241" s="35"/>
       <c r="U241" s="37">
         <f>+F229</f>
-        <v>0.15922031998634348</v>
+        <v>0.15785389542579656</v>
       </c>
       <c r="V241" s="82">
         <f>+F230</f>
-        <v>2.0941400700990314</v>
+        <v>2.0818201462158563</v>
       </c>
     </row>
     <row r="244" spans="2:22" x14ac:dyDescent="0.2">
@@ -7717,27 +7717,27 @@
       </c>
       <c r="E248" s="87">
         <f t="shared" ref="E248:G250" si="43">+(J248)^(365/($R$232-$M$232))-1</f>
-        <v>0.15093470834680933</v>
+        <v>0.14962048020525387</v>
       </c>
       <c r="F248" s="87">
         <f t="shared" si="43"/>
-        <v>0.16877344175968956</v>
+        <v>0.16728101167126863</v>
       </c>
       <c r="G248" s="87">
         <f t="shared" si="43"/>
-        <v>0.19401433253638722</v>
+        <v>0.19228517837747483</v>
       </c>
       <c r="J248" s="88">
         <f t="shared" ref="J248:L250" si="44">+(($R$222+(((($F$164*(1+$D248)*$F$167-$F$172)/$F$163)-$K$167)*$R$216*(1-$K$170))-((E$247-$F$176)*$F$169*(1+5*$F$177*(1-$F$36))))*$F$208)/(($F$164*(1+$D248)*$F$167*$F$168)*(1+$K$168)+$E$202-(E$247*$F$169)-$E$195)</f>
-        <v>2.0203224873704371</v>
+        <v>2.0088076931910432</v>
       </c>
       <c r="K248" s="88">
         <f t="shared" si="44"/>
-        <v>2.1819120210794112</v>
+        <v>2.1680093282379547</v>
       </c>
       <c r="L248" s="88">
         <f t="shared" si="44"/>
-        <v>2.4280559206435202</v>
+        <v>2.4105158221177168</v>
       </c>
       <c r="N248" s="21" t="s">
         <v>216</v>
@@ -7757,27 +7757,27 @@
       </c>
       <c r="E249" s="87">
         <f t="shared" si="43"/>
-        <v>0.14418225215889935</v>
+        <v>0.14296630052020354</v>
       </c>
       <c r="F249" s="90">
         <f t="shared" si="43"/>
-        <v>0.15922032169421341</v>
+        <v>0.15785389946555495</v>
       </c>
       <c r="G249" s="87">
         <f t="shared" si="43"/>
-        <v>0.17973151328233872</v>
+        <v>0.17817049867791046</v>
       </c>
       <c r="J249" s="88">
         <f t="shared" si="44"/>
-        <v>1.9617167293575504</v>
+        <v>1.9513093449405392</v>
       </c>
       <c r="K249" s="91">
         <f t="shared" si="44"/>
-        <v>2.0941400700990318</v>
+        <v>2.0818201462158572</v>
       </c>
       <c r="L249" s="88">
         <f t="shared" si="44"/>
-        <v>2.2861913067879231</v>
+        <v>2.2710976606316486</v>
       </c>
       <c r="N249" s="21" t="s">
         <v>217</v>
@@ -7797,27 +7797,27 @@
       </c>
       <c r="E250" s="87">
         <f t="shared" si="43"/>
-        <v>0.13363061031997003</v>
+        <v>0.1325725576411878</v>
       </c>
       <c r="F250" s="87">
         <f t="shared" si="43"/>
-        <v>0.14484777089315126</v>
+        <v>0.14367814598506645</v>
       </c>
       <c r="G250" s="87">
         <f t="shared" si="43"/>
-        <v>0.15934744044332327</v>
+        <v>0.15803921887792471</v>
       </c>
       <c r="J250" s="88">
         <f t="shared" si="44"/>
-        <v>1.872867521239526</v>
+        <v>1.8641390244230851</v>
       </c>
       <c r="K250" s="88">
         <f t="shared" si="44"/>
-        <v>1.9674317111031394</v>
+        <v>1.9573966863834615</v>
       </c>
       <c r="L250" s="88">
         <f t="shared" si="44"/>
-        <v>2.09528915620634</v>
+        <v>2.0834876137392482</v>
       </c>
       <c r="N250" s="21" t="s">
         <v>218</v>

</xml_diff>